<commit_message>
feat: automatizar ciclo completo de consulta e salvar em organização pré-definida
</commit_message>
<xml_diff>
--- a/usuario-senha-nfe.xlsx
+++ b/usuario-senha-nfe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Setor Administrativo\Documents\consulta-nfe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648D0CEF-C2CA-42FA-875F-AE6706DB90A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8517F094-BF27-43E7-B276-CAF78F30E611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>RAZÃO SOCIAL</t>
   </si>
@@ -41,6 +41,18 @@
   </si>
   <si>
     <t>con2686</t>
+  </si>
+  <si>
+    <t>RIOS DELICATESSEN LTDA</t>
+  </si>
+  <si>
+    <t>08.385.805/0001-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7239626900	</t>
+  </si>
+  <si>
+    <t>con0595</t>
   </si>
 </sst>
 </file>
@@ -50,7 +62,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[&lt;=99999999999]000\.000\.000\-00;00\.000\.000\/0000\-00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -80,8 +92,14 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -106,8 +124,14 @@
         <bgColor rgb="FF00427A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -130,11 +154,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -149,6 +199,12 @@
     </xf>
     <xf numFmtId="1" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -233,7 +289,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:D2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:D3">
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="RAZÃO SOCIAL"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="CNPJ" dataDxfId="2"/>
@@ -467,7 +523,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -481,88 +537,97 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
+      <c r="C4" s="6"/>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
+      <c r="C5" s="6"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
+      <c r="C6" s="6"/>
       <c r="D6" s="4"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
+      <c r="C7" s="6"/>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
+      <c r="C8" s="6"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
+      <c r="C9" s="6"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
+      <c r="C10" s="6"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
+      <c r="C11" s="6"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
+      <c r="C12" s="6"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
+      <c r="C13" s="6"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
+      <c r="C14" s="6"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
+      <c r="C15" s="6"/>
       <c r="D15" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adição de função para download de destinatários e atualização no funcionamento do OCR
</commit_message>
<xml_diff>
--- a/usuario-senha-nfe.xlsx
+++ b/usuario-senha-nfe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Setor Administrativo\Documents\consulta-nfe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8517F094-BF27-43E7-B276-CAF78F30E611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62193848-BBB4-463F-908B-248CE58A7634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Página1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>RAZÃO SOCIAL</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t>con0595</t>
+  </si>
+  <si>
+    <t>CÓDIGO DOMINIO</t>
   </si>
 </sst>
 </file>
@@ -189,28 +192,49 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="8">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00427A"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
       <fill>
@@ -219,6 +243,7 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border outline="0">
         <right style="thin">
           <color rgb="FF000000"/>
@@ -226,24 +251,15 @@
       </border>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF00427A"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-      </border>
-    </dxf>
-    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border outline="0">
         <right style="thin">
           <color rgb="FF000000"/>
         </right>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -272,9 +288,9 @@
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Página1-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="firstRowStripe" dxfId="4"/>
-      <tableStyleElement type="secondRowStripe" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+      <tableStyleElement type="firstRowStripe" dxfId="6"/>
+      <tableStyleElement type="secondRowStripe" dxfId="5"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -289,11 +305,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:D3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="B1:E3" dataDxfId="0">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="RAZÃO SOCIAL"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="CNPJ" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="usuario" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="RAZÃO SOCIAL" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="CNPJ" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="usuario" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="senha" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="Página1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
@@ -501,127 +517,149 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="38.42578125" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="38.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>2686</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="6">
+      <c r="D2" s="6">
         <v>5782014300</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>595</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="4"/>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="8"/>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="8"/>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="8"/>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="8"/>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="8"/>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="8"/>
+    </row>
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="8"/>
+    </row>
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="8"/>
+    </row>
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="8"/>
+    </row>
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="8"/>
+    </row>
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="8"/>
+    </row>
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>